<commit_message>
vault backup: 2026-10-19 10:35:51
</commit_message>
<xml_diff>
--- a/Procurement/_документы/План закупок Таза – IV кв. 2026.xlsx
+++ b/Procurement/_документы/План закупок Таза – IV кв. 2026.xlsx
@@ -5,11 +5,11 @@
   <workbookPr defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Закупки\1 Процедуры закупок\2 План закупок\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Obsidian\Procurement\_документы\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="21570" windowHeight="10125"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="21570" windowHeight="10125" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Свод" sheetId="3" r:id="rId1"/>
@@ -34,9 +34,6 @@
     <t>ЧФ "Central Asia Climate Foundation"</t>
   </si>
   <si>
-    <t>План закупок товаров, работ и неконсультационных услуг проектного офиса «Таза Қазақстан» на IV квартал 2026 года</t>
-  </si>
-  <si>
     <t>БИН: 240240900538</t>
   </si>
   <si>
@@ -592,9 +589,6 @@
     <t>Аутсорс</t>
   </si>
   <si>
-    <t>Системное администрирование (аутсорс)</t>
-  </si>
-  <si>
     <t>Разработка ИИ- и ГИС-инструментов, цифровой платформы (аутсорс)</t>
   </si>
   <si>
@@ -898,12 +892,6 @@
     <t>Дизайн визуалов, инфографики и презентаций – 2 лицензии.</t>
   </si>
   <si>
-    <t>Видео-конференц-связь с регионами – 2 лицензии.</t>
-  </si>
-  <si>
-    <t>Договоры и соглашения, право МФЦА, сопровождение закупок и кадровых документов – с 21.10.2026, 2,35 месяца по 1 160 000 ₸.</t>
-  </si>
-  <si>
     <t>ИТ-инфраструктура, сеть и техника; делопроизводство, хозяйственное администрирование, ассистирование – с 21.10.2026, 2,35 месяца по 812 000 ₸.</t>
   </si>
   <si>
@@ -932,6 +920,18 @@
   </si>
   <si>
     <t>Универсальное моющее средство "Yarko", 5 л – 3 395 ₸; "Mr.Proper", Лимон, 5 л – 8 335 ₸</t>
+  </si>
+  <si>
+    <t>План закупок товаров, работ и неконсультационных услуг на IV квартал 2026 года</t>
+  </si>
+  <si>
+    <t>Видео-конференц-связь с регионами – лицензия.</t>
+  </si>
+  <si>
+    <t>Договоры и соглашения, право МФЦА – с 21.10.2026, 2,35 месяца по 1 160 000 ₸.</t>
+  </si>
+  <si>
+    <t>Администрирование (аутсорс)</t>
   </si>
 </sst>
 </file>
@@ -983,7 +983,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -993,6 +993,24 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFE2EFDA"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.39997558519241921"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1033,7 +1051,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1080,6 +1098,9 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
@@ -1089,8 +1110,17 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1383,31 +1413,31 @@
   <sheetData>
     <row r="1" spans="1:6" ht="17.25" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="45" x14ac:dyDescent="0.25">
       <c r="A4" s="10" t="s">
+        <v>113</v>
+      </c>
+      <c r="B4" s="10" t="s">
         <v>114</v>
       </c>
-      <c r="B4" s="10" t="s">
+      <c r="C4" s="10" t="s">
         <v>115</v>
       </c>
-      <c r="C4" s="10" t="s">
-        <v>116</v>
-      </c>
-      <c r="D4" s="23"/>
-      <c r="E4" s="23"/>
-      <c r="F4" s="23"/>
+      <c r="D4" s="18"/>
+      <c r="E4" s="18"/>
+      <c r="F4" s="18"/>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="15" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="B5" s="16">
         <v>58691748</v>
@@ -1421,7 +1451,7 @@
     </row>
     <row r="6" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A6" s="15" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="B6" s="16">
         <v>14567355</v>
@@ -1436,7 +1466,7 @@
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="15" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="B7" s="16">
         <v>500000</v>
@@ -1451,7 +1481,7 @@
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="15" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="B8" s="16">
         <v>3783804</v>
@@ -1466,7 +1496,7 @@
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="15" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="B9" s="16">
         <v>29170035</v>
@@ -1481,7 +1511,7 @@
     </row>
     <row r="10" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A10" s="15" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="B10" s="16">
         <v>17530038</v>
@@ -1496,7 +1526,7 @@
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="15" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="B11" s="16">
         <v>589500</v>
@@ -1511,7 +1541,7 @@
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="15" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="B12" s="16">
         <v>2525000</v>
@@ -1526,7 +1556,7 @@
     </row>
     <row r="13" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A13" s="15" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="B13" s="16">
         <v>12810748</v>
@@ -1541,7 +1571,7 @@
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="15" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="B14" s="16">
         <v>87404855</v>
@@ -1556,7 +1586,7 @@
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="13" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B15" s="14">
         <f>SUM(B5:B14)</f>
@@ -1572,7 +1602,7 @@
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="15" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="B16" s="16"/>
       <c r="C16" s="16">
@@ -2008,32 +2038,32 @@
       <c r="H3" s="2"/>
       <c r="I3" s="2"/>
       <c r="J3" s="2" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="K3" s="2"/>
       <c r="L3" s="2"/>
       <c r="M3" s="2"/>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A4" s="18" t="s">
-        <v>2</v>
-      </c>
-      <c r="B4" s="19"/>
-      <c r="C4" s="19"/>
-      <c r="D4" s="19"/>
-      <c r="E4" s="19"/>
-      <c r="F4" s="19"/>
-      <c r="G4" s="19"/>
-      <c r="H4" s="19"/>
-      <c r="I4" s="19"/>
-      <c r="J4" s="19"/>
-      <c r="K4" s="19"/>
-      <c r="L4" s="19"/>
-      <c r="M4" s="19"/>
+      <c r="A4" s="19" t="s">
+        <v>298</v>
+      </c>
+      <c r="B4" s="20"/>
+      <c r="C4" s="20"/>
+      <c r="D4" s="20"/>
+      <c r="E4" s="20"/>
+      <c r="F4" s="20"/>
+      <c r="G4" s="20"/>
+      <c r="H4" s="20"/>
+      <c r="I4" s="20"/>
+      <c r="J4" s="20"/>
+      <c r="K4" s="20"/>
+      <c r="L4" s="20"/>
+      <c r="M4" s="20"/>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B5" s="2"/>
       <c r="C5" s="2"/>
@@ -2049,25 +2079,25 @@
       <c r="M5" s="2"/>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A6" s="20" t="s">
-        <v>4</v>
-      </c>
-      <c r="B6" s="19"/>
-      <c r="C6" s="19"/>
-      <c r="D6" s="19"/>
-      <c r="E6" s="19"/>
-      <c r="F6" s="19"/>
-      <c r="G6" s="19"/>
-      <c r="H6" s="19"/>
-      <c r="I6" s="19"/>
-      <c r="J6" s="19"/>
-      <c r="K6" s="19"/>
-      <c r="L6" s="19"/>
-      <c r="M6" s="19"/>
+      <c r="A6" s="21" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" s="20"/>
+      <c r="C6" s="20"/>
+      <c r="D6" s="20"/>
+      <c r="E6" s="20"/>
+      <c r="F6" s="20"/>
+      <c r="G6" s="20"/>
+      <c r="H6" s="20"/>
+      <c r="I6" s="20"/>
+      <c r="J6" s="20"/>
+      <c r="K6" s="20"/>
+      <c r="L6" s="20"/>
+      <c r="M6" s="20"/>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -2083,61 +2113,61 @@
       <c r="M7" s="2"/>
     </row>
     <row r="8" spans="1:13" ht="45.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="21" t="s">
-        <v>263</v>
-      </c>
-      <c r="B8" s="22"/>
-      <c r="C8" s="22"/>
-      <c r="D8" s="22"/>
-      <c r="E8" s="22"/>
-      <c r="F8" s="22"/>
-      <c r="G8" s="22"/>
-      <c r="H8" s="22"/>
-      <c r="I8" s="22"/>
-      <c r="J8" s="22"/>
-      <c r="K8" s="22"/>
-      <c r="L8" s="22"/>
-      <c r="M8" s="22"/>
+      <c r="A8" s="22" t="s">
+        <v>261</v>
+      </c>
+      <c r="B8" s="23"/>
+      <c r="C8" s="23"/>
+      <c r="D8" s="23"/>
+      <c r="E8" s="23"/>
+      <c r="F8" s="23"/>
+      <c r="G8" s="23"/>
+      <c r="H8" s="23"/>
+      <c r="I8" s="23"/>
+      <c r="J8" s="23"/>
+      <c r="K8" s="23"/>
+      <c r="L8" s="23"/>
+      <c r="M8" s="23"/>
     </row>
     <row r="9" spans="1:13" ht="57.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B9" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="B9" s="3" t="s">
+      <c r="C9" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="D9" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="D9" s="3" t="s">
+      <c r="E9" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="E9" s="3" t="s">
+      <c r="F9" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="F9" s="3" t="s">
+      <c r="G9" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="G9" s="3" t="s">
+      <c r="H9" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="H9" s="3" t="s">
+      <c r="I9" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="I9" s="3" t="s">
+      <c r="J9" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="J9" s="3" t="s">
+      <c r="K9" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="K9" s="3" t="s">
+      <c r="L9" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="L9" s="3" t="s">
+      <c r="M9" s="3" t="s">
         <v>16</v>
-      </c>
-      <c r="M9" s="3" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.25">
@@ -2189,16 +2219,16 @@
         <v>1</v>
       </c>
       <c r="C11" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="D11" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="D11" s="5" t="s">
+      <c r="E11" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="E11" s="5" t="s">
+      <c r="F11" s="8" t="s">
         <v>20</v>
-      </c>
-      <c r="F11" s="8" t="s">
-        <v>21</v>
       </c>
       <c r="G11" s="6">
         <v>12</v>
@@ -2207,20 +2237,20 @@
         <v>522000</v>
       </c>
       <c r="I11" s="6">
-        <f>ROUND(G11*H11,0)</f>
+        <f t="shared" ref="I11:I42" si="0">ROUND(G11*H11,0)</f>
         <v>6264000</v>
       </c>
       <c r="J11" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="K11" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="K11" s="5" t="s">
-        <v>23</v>
-      </c>
       <c r="L11" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="M11" s="5" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="12" spans="1:13" ht="45" x14ac:dyDescent="0.25">
@@ -2231,16 +2261,16 @@
         <v>2</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="F12" s="8" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G12" s="6">
         <v>2</v>
@@ -2249,20 +2279,20 @@
         <v>1044000</v>
       </c>
       <c r="I12" s="6">
-        <f>ROUND(G12*H12,0)</f>
+        <f t="shared" si="0"/>
         <v>2088000</v>
       </c>
       <c r="J12" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="K12" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="K12" s="5" t="s">
-        <v>23</v>
-      </c>
       <c r="L12" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="M12" s="5" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="13" spans="1:13" ht="30" x14ac:dyDescent="0.25">
@@ -2273,16 +2303,16 @@
         <v>3</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D13" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="E13" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="E13" s="5" t="s">
-        <v>27</v>
-      </c>
       <c r="F13" s="8" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G13" s="6">
         <v>10</v>
@@ -2291,20 +2321,20 @@
         <v>116000</v>
       </c>
       <c r="I13" s="6">
-        <f>ROUND(G13*H13,0)</f>
+        <f t="shared" si="0"/>
         <v>1160000</v>
       </c>
       <c r="J13" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="K13" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="K13" s="5" t="s">
-        <v>23</v>
-      </c>
       <c r="L13" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="M13" s="5" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="14" spans="1:13" ht="45" x14ac:dyDescent="0.25">
@@ -2315,16 +2345,16 @@
         <v>4</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D14" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="E14" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="E14" s="5" t="s">
-        <v>29</v>
-      </c>
       <c r="F14" s="8" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G14" s="6">
         <v>19</v>
@@ -2333,20 +2363,20 @@
         <v>232000</v>
       </c>
       <c r="I14" s="6">
-        <f>ROUND(G14*H14,0)</f>
+        <f t="shared" si="0"/>
         <v>4408000</v>
       </c>
       <c r="J14" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="K14" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="K14" s="5" t="s">
-        <v>23</v>
-      </c>
       <c r="L14" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="M14" s="5" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="15" spans="1:13" ht="45" x14ac:dyDescent="0.25">
@@ -2357,16 +2387,16 @@
         <v>5</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E15" s="5" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="F15" s="8" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G15" s="6">
         <v>5</v>
@@ -2375,20 +2405,20 @@
         <v>580000</v>
       </c>
       <c r="I15" s="6">
-        <f>ROUND(G15*H15,0)</f>
+        <f t="shared" si="0"/>
         <v>2900000</v>
       </c>
       <c r="J15" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="K15" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="K15" s="5" t="s">
-        <v>23</v>
-      </c>
       <c r="L15" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="M15" s="5" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="16" spans="1:13" ht="30" x14ac:dyDescent="0.25">
@@ -2399,16 +2429,16 @@
         <v>6</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D16" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="E16" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="E16" s="5" t="s">
-        <v>33</v>
-      </c>
       <c r="F16" s="8" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G16" s="6">
         <v>1</v>
@@ -2417,20 +2447,20 @@
         <v>928000</v>
       </c>
       <c r="I16" s="6">
-        <f>ROUND(G16*H16,0)</f>
+        <f t="shared" si="0"/>
         <v>928000</v>
       </c>
       <c r="J16" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="K16" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="K16" s="5" t="s">
-        <v>23</v>
-      </c>
       <c r="L16" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="M16" s="5" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.25">
@@ -2441,16 +2471,16 @@
         <v>7</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="F17" s="8" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G17" s="6">
         <v>1</v>
@@ -2459,20 +2489,20 @@
         <v>290000</v>
       </c>
       <c r="I17" s="6">
-        <f>ROUND(G17*H17,0)</f>
+        <f t="shared" si="0"/>
         <v>290000</v>
       </c>
       <c r="J17" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="K17" s="5" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="L17" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="M17" s="5" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="18" spans="1:13" ht="30" x14ac:dyDescent="0.25">
@@ -2483,16 +2513,16 @@
         <v>8</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E18" s="5" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="F18" s="8" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G18" s="6">
         <v>1</v>
@@ -2501,20 +2531,20 @@
         <v>522000</v>
       </c>
       <c r="I18" s="6">
-        <f>ROUND(G18*H18,0)</f>
+        <f t="shared" si="0"/>
         <v>522000</v>
       </c>
       <c r="J18" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="K18" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="K18" s="5" t="s">
-        <v>23</v>
-      </c>
       <c r="L18" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="M18" s="5" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="19" spans="1:13" ht="30" x14ac:dyDescent="0.25">
@@ -2525,16 +2555,16 @@
         <v>9</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D19" s="5" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="E19" s="5" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="F19" s="8" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G19" s="6">
         <v>2</v>
@@ -2543,20 +2573,20 @@
         <v>69600</v>
       </c>
       <c r="I19" s="6">
-        <f>ROUND(G19*H19,0)</f>
+        <f t="shared" si="0"/>
         <v>139200</v>
       </c>
       <c r="J19" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="K19" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="K19" s="5" t="s">
-        <v>23</v>
-      </c>
       <c r="L19" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="M19" s="5" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="20" spans="1:13" ht="45" x14ac:dyDescent="0.25">
@@ -2567,16 +2597,16 @@
         <v>10</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="E20" s="5" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="F20" s="8" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G20" s="6">
         <v>1</v>
@@ -2585,20 +2615,20 @@
         <v>918720</v>
       </c>
       <c r="I20" s="6">
-        <f>ROUND(G20*H20,0)</f>
+        <f t="shared" si="0"/>
         <v>918720</v>
       </c>
       <c r="J20" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="K20" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="K20" s="5" t="s">
-        <v>23</v>
-      </c>
       <c r="L20" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="M20" s="5" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="21" spans="1:13" ht="45" x14ac:dyDescent="0.25">
@@ -2609,16 +2639,16 @@
         <v>11</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D21" s="5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E21" s="5" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="F21" s="8" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G21" s="6">
         <v>1</v>
@@ -2627,20 +2657,20 @@
         <v>2900000</v>
       </c>
       <c r="I21" s="6">
-        <f>ROUND(G21*H21,0)</f>
+        <f t="shared" si="0"/>
         <v>2900000</v>
       </c>
       <c r="J21" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="K21" s="5" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="L21" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="M21" s="5" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="22" spans="1:13" ht="30" x14ac:dyDescent="0.25">
@@ -2651,16 +2681,16 @@
         <v>12</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D22" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="E22" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="E22" s="5" t="s">
-        <v>38</v>
-      </c>
       <c r="F22" s="8" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G22" s="6">
         <v>2</v>
@@ -2669,20 +2699,20 @@
         <v>348000</v>
       </c>
       <c r="I22" s="6">
-        <f>ROUND(G22*H22,0)</f>
+        <f t="shared" si="0"/>
         <v>696000</v>
       </c>
       <c r="J22" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="K22" s="5" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="L22" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="M22" s="5" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="23" spans="1:13" ht="60" x14ac:dyDescent="0.25">
@@ -2693,16 +2723,16 @@
         <v>13</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D23" s="5" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E23" s="5" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="F23" s="8" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G23" s="6">
         <v>2</v>
@@ -2711,20 +2741,20 @@
         <v>324800</v>
       </c>
       <c r="I23" s="6">
-        <f>ROUND(G23*H23,0)</f>
+        <f t="shared" si="0"/>
         <v>649600</v>
       </c>
       <c r="J23" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="K23" s="5" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="L23" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="M23" s="5" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="24" spans="1:13" ht="30" x14ac:dyDescent="0.25">
@@ -2735,16 +2765,16 @@
         <v>14</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D24" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="E24" s="5" t="s">
+        <v>276</v>
+      </c>
+      <c r="F24" s="8" t="s">
         <v>40</v>
-      </c>
-      <c r="E24" s="5" t="s">
-        <v>278</v>
-      </c>
-      <c r="F24" s="8" t="s">
-        <v>41</v>
       </c>
       <c r="G24" s="6">
         <v>4</v>
@@ -2753,20 +2783,20 @@
         <v>63800</v>
       </c>
       <c r="I24" s="6">
-        <f>ROUND(G24*H24,0)</f>
+        <f t="shared" si="0"/>
         <v>255200</v>
       </c>
       <c r="J24" s="5" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="K24" s="5" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="L24" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="M24" s="5" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="25" spans="1:13" ht="30" x14ac:dyDescent="0.25">
@@ -2777,16 +2807,16 @@
         <v>15</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D25" s="5" t="s">
+        <v>167</v>
+      </c>
+      <c r="E25" s="5" t="s">
         <v>168</v>
       </c>
-      <c r="E25" s="5" t="s">
-        <v>169</v>
-      </c>
       <c r="F25" s="8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="G25" s="6">
         <v>1</v>
@@ -2795,20 +2825,20 @@
         <v>42340</v>
       </c>
       <c r="I25" s="6">
-        <f>ROUND(G25*H25,0)</f>
+        <f t="shared" si="0"/>
         <v>42340</v>
       </c>
       <c r="J25" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="K25" s="5" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="L25" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="M25" s="5" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="26" spans="1:13" ht="30" x14ac:dyDescent="0.25">
@@ -2819,16 +2849,16 @@
         <v>16</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D26" s="5" t="s">
+        <v>170</v>
+      </c>
+      <c r="E26" s="5" t="s">
         <v>171</v>
       </c>
-      <c r="E26" s="5" t="s">
-        <v>172</v>
-      </c>
       <c r="F26" s="8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="G26" s="6">
         <v>1</v>
@@ -2837,20 +2867,20 @@
         <v>6000</v>
       </c>
       <c r="I26" s="6">
-        <f>ROUND(G26*H26,0)</f>
+        <f t="shared" si="0"/>
         <v>6000</v>
       </c>
       <c r="J26" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="K26" s="5" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="L26" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="M26" s="5" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="27" spans="1:13" ht="30" x14ac:dyDescent="0.25">
@@ -2861,16 +2891,16 @@
         <v>17</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D27" s="5" t="s">
+        <v>172</v>
+      </c>
+      <c r="E27" s="5" t="s">
         <v>173</v>
       </c>
-      <c r="E27" s="5" t="s">
-        <v>174</v>
-      </c>
       <c r="F27" s="8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="G27" s="6">
         <v>1</v>
@@ -2879,20 +2909,20 @@
         <v>114327</v>
       </c>
       <c r="I27" s="6">
-        <f>ROUND(G27*H27,0)</f>
+        <f t="shared" si="0"/>
         <v>114327</v>
       </c>
       <c r="J27" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="K27" s="5" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="L27" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="M27" s="5" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="28" spans="1:13" ht="30" x14ac:dyDescent="0.25">
@@ -2903,16 +2933,16 @@
         <v>18</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D28" s="5" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="E28" s="5" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="F28" s="8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="G28" s="6">
         <v>1</v>
@@ -2921,20 +2951,20 @@
         <v>48700</v>
       </c>
       <c r="I28" s="6">
-        <f>ROUND(G28*H28,0)</f>
+        <f t="shared" si="0"/>
         <v>48700</v>
       </c>
       <c r="J28" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="K28" s="5" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="L28" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="M28" s="5" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
     </row>
     <row r="29" spans="1:13" ht="45" x14ac:dyDescent="0.25">
@@ -2945,16 +2975,16 @@
         <v>19</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D29" s="5" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="E29" s="5" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="F29" s="8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="G29" s="6">
         <v>1</v>
@@ -2963,20 +2993,20 @@
         <v>989997</v>
       </c>
       <c r="I29" s="6">
-        <f>ROUND(G29*H29,0)</f>
+        <f t="shared" si="0"/>
         <v>989997</v>
       </c>
       <c r="J29" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="K29" s="5" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="L29" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="M29" s="5" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
     </row>
     <row r="30" spans="1:13" ht="30" x14ac:dyDescent="0.25">
@@ -2987,16 +3017,16 @@
         <v>20</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D30" s="5" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="E30" s="5" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="F30" s="8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="G30" s="6">
         <v>1</v>
@@ -3005,20 +3035,20 @@
         <v>49990</v>
       </c>
       <c r="I30" s="6">
-        <f>ROUND(G30*H30,0)</f>
+        <f t="shared" si="0"/>
         <v>49990</v>
       </c>
       <c r="J30" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="K30" s="5" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="L30" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="M30" s="5" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
     </row>
     <row r="31" spans="1:13" ht="30" x14ac:dyDescent="0.25">
@@ -3029,16 +3059,16 @@
         <v>21</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D31" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="E31" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="E31" s="5" t="s">
-        <v>44</v>
-      </c>
       <c r="F31" s="8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="G31" s="6">
         <v>1</v>
@@ -3047,20 +3077,20 @@
         <v>348000</v>
       </c>
       <c r="I31" s="6">
-        <f>ROUND(G31*H31,0)</f>
+        <f t="shared" si="0"/>
         <v>348000</v>
       </c>
       <c r="J31" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="K31" s="5" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="L31" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="M31" s="5" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="32" spans="1:13" ht="45" x14ac:dyDescent="0.25">
@@ -3071,16 +3101,16 @@
         <v>22</v>
       </c>
       <c r="C32" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="D32" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="D32" s="5" t="s">
-        <v>46</v>
-      </c>
       <c r="E32" s="5" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="F32" s="8" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G32" s="6">
         <v>1</v>
@@ -3089,20 +3119,20 @@
         <v>928000</v>
       </c>
       <c r="I32" s="6">
-        <f>ROUND(G32*H32,0)</f>
+        <f t="shared" si="0"/>
         <v>928000</v>
       </c>
       <c r="J32" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="K32" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="K32" s="5" t="s">
-        <v>23</v>
-      </c>
       <c r="L32" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="M32" s="5" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="33" spans="1:13" ht="30" x14ac:dyDescent="0.25">
@@ -3113,16 +3143,16 @@
         <v>23</v>
       </c>
       <c r="C33" s="5" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D33" s="5" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E33" s="5" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="F33" s="8" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G33" s="6">
         <v>1</v>
@@ -3131,20 +3161,20 @@
         <v>812000</v>
       </c>
       <c r="I33" s="6">
-        <f>ROUND(G33*H33,0)</f>
+        <f t="shared" si="0"/>
         <v>812000</v>
       </c>
       <c r="J33" s="5" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="K33" s="5" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="L33" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="M33" s="5" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="34" spans="1:13" ht="45" x14ac:dyDescent="0.25">
@@ -3155,16 +3185,16 @@
         <v>24</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D34" s="5" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E34" s="5" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="F34" s="8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="G34" s="6">
         <v>16</v>
@@ -3173,20 +3203,20 @@
         <v>4118</v>
       </c>
       <c r="I34" s="6">
-        <f>ROUND(G34*H34,0)</f>
+        <f t="shared" si="0"/>
         <v>65888</v>
       </c>
       <c r="J34" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="K34" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="K34" s="5" t="s">
-        <v>23</v>
-      </c>
       <c r="L34" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="M34" s="5" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="35" spans="1:13" ht="30" x14ac:dyDescent="0.25">
@@ -3197,16 +3227,16 @@
         <v>25</v>
       </c>
       <c r="C35" s="5" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D35" s="5" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="E35" s="5" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="F35" s="8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="G35" s="6">
         <v>3</v>
@@ -3215,20 +3245,20 @@
         <v>6101</v>
       </c>
       <c r="I35" s="6">
-        <f>ROUND(G35*H35,0)</f>
+        <f t="shared" si="0"/>
         <v>18303</v>
       </c>
       <c r="J35" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="K35" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="K35" s="5" t="s">
-        <v>23</v>
-      </c>
       <c r="L35" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="M35" s="5" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="36" spans="1:13" ht="30" x14ac:dyDescent="0.25">
@@ -3239,16 +3269,16 @@
         <v>26</v>
       </c>
       <c r="C36" s="5" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D36" s="5" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="E36" s="5" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="F36" s="8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="G36" s="6">
         <v>4</v>
@@ -3257,20 +3287,20 @@
         <v>7235</v>
       </c>
       <c r="I36" s="6">
-        <f>ROUND(G36*H36,0)</f>
+        <f t="shared" si="0"/>
         <v>28940</v>
       </c>
       <c r="J36" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="K36" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="K36" s="5" t="s">
-        <v>23</v>
-      </c>
       <c r="L36" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="M36" s="5" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
     </row>
     <row r="37" spans="1:13" ht="30" x14ac:dyDescent="0.25">
@@ -3281,16 +3311,16 @@
         <v>27</v>
       </c>
       <c r="C37" s="5" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D37" s="5" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="E37" s="5" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="F37" s="8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="G37" s="6">
         <v>5</v>
@@ -3299,20 +3329,20 @@
         <v>9039</v>
       </c>
       <c r="I37" s="6">
-        <f>ROUND(G37*H37,0)</f>
+        <f t="shared" si="0"/>
         <v>45195</v>
       </c>
       <c r="J37" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="K37" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="K37" s="5" t="s">
-        <v>23</v>
-      </c>
       <c r="L37" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="M37" s="5" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
     </row>
     <row r="38" spans="1:13" ht="45" x14ac:dyDescent="0.25">
@@ -3323,16 +3353,16 @@
         <v>28</v>
       </c>
       <c r="C38" s="5" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D38" s="5" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="E38" s="5" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="F38" s="8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="G38" s="6">
         <v>10</v>
@@ -3341,20 +3371,20 @@
         <v>89302</v>
       </c>
       <c r="I38" s="6">
-        <f>ROUND(G38*H38,0)</f>
+        <f t="shared" si="0"/>
         <v>893020</v>
       </c>
       <c r="J38" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="K38" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="K38" s="5" t="s">
-        <v>23</v>
-      </c>
       <c r="L38" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="M38" s="5" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
     </row>
     <row r="39" spans="1:13" ht="45" x14ac:dyDescent="0.25">
@@ -3365,16 +3395,16 @@
         <v>29</v>
       </c>
       <c r="C39" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="D39" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="D39" s="24" t="s">
+        <v>47</v>
+      </c>
+      <c r="E39" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="E39" s="5" t="s">
-        <v>49</v>
-      </c>
       <c r="F39" s="8" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G39" s="6">
         <v>1</v>
@@ -3383,20 +3413,20 @@
         <v>1669990</v>
       </c>
       <c r="I39" s="6">
-        <f>ROUND(G39*H39,0)</f>
+        <f t="shared" si="0"/>
         <v>1669990</v>
       </c>
       <c r="J39" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="K39" s="5" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="L39" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="M39" s="5" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
     </row>
     <row r="40" spans="1:13" ht="30" x14ac:dyDescent="0.25">
@@ -3407,16 +3437,16 @@
         <v>30</v>
       </c>
       <c r="C40" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="D40" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="D40" s="24" t="s">
+        <v>49</v>
+      </c>
+      <c r="E40" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="E40" s="5" t="s">
-        <v>51</v>
-      </c>
       <c r="F40" s="8" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G40" s="6">
         <v>1</v>
@@ -3425,20 +3455,20 @@
         <v>485990</v>
       </c>
       <c r="I40" s="6">
-        <f>ROUND(G40*H40,0)</f>
+        <f t="shared" si="0"/>
         <v>485990</v>
       </c>
       <c r="J40" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="K40" s="5" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="L40" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="M40" s="5" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
     </row>
     <row r="41" spans="1:13" ht="30" x14ac:dyDescent="0.25">
@@ -3449,16 +3479,16 @@
         <v>31</v>
       </c>
       <c r="C41" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="D41" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="D41" s="24" t="s">
+        <v>51</v>
+      </c>
+      <c r="E41" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="E41" s="5" t="s">
-        <v>53</v>
-      </c>
       <c r="F41" s="8" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G41" s="6">
         <v>1</v>
@@ -3467,20 +3497,20 @@
         <v>479990</v>
       </c>
       <c r="I41" s="6">
-        <f>ROUND(G41*H41,0)</f>
+        <f t="shared" si="0"/>
         <v>479990</v>
       </c>
       <c r="J41" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="K41" s="5" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="L41" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="M41" s="5" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
     </row>
     <row r="42" spans="1:13" ht="30" x14ac:dyDescent="0.25">
@@ -3491,16 +3521,16 @@
         <v>32</v>
       </c>
       <c r="C42" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="D42" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="D42" s="24" t="s">
+        <v>53</v>
+      </c>
+      <c r="E42" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="E42" s="5" t="s">
-        <v>55</v>
-      </c>
       <c r="F42" s="8" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G42" s="6">
         <v>1</v>
@@ -3509,20 +3539,20 @@
         <v>58990</v>
       </c>
       <c r="I42" s="6">
-        <f>ROUND(G42*H42,0)</f>
+        <f t="shared" si="0"/>
         <v>58990</v>
       </c>
       <c r="J42" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="K42" s="5" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="L42" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="M42" s="5" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
     </row>
     <row r="43" spans="1:13" ht="30" x14ac:dyDescent="0.25">
@@ -3533,16 +3563,16 @@
         <v>33</v>
       </c>
       <c r="C43" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="D43" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="D43" s="24" t="s">
+        <v>55</v>
+      </c>
+      <c r="E43" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="E43" s="5" t="s">
-        <v>57</v>
-      </c>
       <c r="F43" s="8" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G43" s="6">
         <v>1</v>
@@ -3551,20 +3581,20 @@
         <v>250000</v>
       </c>
       <c r="I43" s="6">
-        <f>ROUND(G43*H43,0)</f>
+        <f t="shared" ref="I43:I74" si="1">ROUND(G43*H43,0)</f>
         <v>250000</v>
       </c>
       <c r="J43" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="K43" s="5" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="L43" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="M43" s="5" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
     </row>
     <row r="44" spans="1:13" ht="30" x14ac:dyDescent="0.25">
@@ -3575,16 +3605,16 @@
         <v>34</v>
       </c>
       <c r="C44" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="D44" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="D44" s="24" t="s">
+        <v>57</v>
+      </c>
+      <c r="E44" s="5" t="s">
         <v>58</v>
       </c>
-      <c r="E44" s="5" t="s">
-        <v>59</v>
-      </c>
       <c r="F44" s="8" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G44" s="6">
         <v>1</v>
@@ -3593,20 +3623,20 @@
         <v>31990</v>
       </c>
       <c r="I44" s="6">
-        <f>ROUND(G44*H44,0)</f>
+        <f t="shared" si="1"/>
         <v>31990</v>
       </c>
       <c r="J44" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="K44" s="5" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="L44" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="M44" s="5" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
     </row>
     <row r="45" spans="1:13" ht="45" x14ac:dyDescent="0.25">
@@ -3617,16 +3647,16 @@
         <v>35</v>
       </c>
       <c r="C45" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="D45" s="5" t="s">
-        <v>60</v>
+        <v>17</v>
+      </c>
+      <c r="D45" s="24" t="s">
+        <v>59</v>
       </c>
       <c r="E45" s="5" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="F45" s="8" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G45" s="6">
         <v>1</v>
@@ -3635,20 +3665,20 @@
         <v>119990</v>
       </c>
       <c r="I45" s="6">
-        <f>ROUND(G45*H45,0)</f>
+        <f t="shared" si="1"/>
         <v>119990</v>
       </c>
       <c r="J45" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="K45" s="5" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="L45" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="M45" s="5" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
     </row>
     <row r="46" spans="1:13" ht="30" x14ac:dyDescent="0.25">
@@ -3659,16 +3689,16 @@
         <v>36</v>
       </c>
       <c r="C46" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="D46" s="5" t="s">
-        <v>61</v>
+        <v>17</v>
+      </c>
+      <c r="D46" s="24" t="s">
+        <v>60</v>
       </c>
       <c r="E46" s="5" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="F46" s="8" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G46" s="6">
         <v>1</v>
@@ -3677,20 +3707,20 @@
         <v>104990</v>
       </c>
       <c r="I46" s="6">
-        <f>ROUND(G46*H46,0)</f>
+        <f t="shared" si="1"/>
         <v>104990</v>
       </c>
       <c r="J46" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="K46" s="5" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="L46" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="M46" s="5" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
     </row>
     <row r="47" spans="1:13" ht="30" x14ac:dyDescent="0.25">
@@ -3701,16 +3731,16 @@
         <v>37</v>
       </c>
       <c r="C47" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="D47" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="D47" s="24" t="s">
+        <v>61</v>
+      </c>
+      <c r="E47" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="E47" s="5" t="s">
-        <v>63</v>
-      </c>
       <c r="F47" s="8" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G47" s="6">
         <v>1</v>
@@ -3719,20 +3749,20 @@
         <v>150000</v>
       </c>
       <c r="I47" s="6">
-        <f>ROUND(G47*H47,0)</f>
+        <f t="shared" si="1"/>
         <v>150000</v>
       </c>
       <c r="J47" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="K47" s="5" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="L47" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="M47" s="5" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
     </row>
     <row r="48" spans="1:13" ht="30" x14ac:dyDescent="0.25">
@@ -3743,16 +3773,16 @@
         <v>38</v>
       </c>
       <c r="C48" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="D48" s="5" t="s">
-        <v>64</v>
+        <v>17</v>
+      </c>
+      <c r="D48" s="24" t="s">
+        <v>63</v>
       </c>
       <c r="E48" s="5" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="F48" s="8" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G48" s="6">
         <v>1</v>
@@ -3761,20 +3791,20 @@
         <v>240000</v>
       </c>
       <c r="I48" s="6">
-        <f>ROUND(G48*H48,0)</f>
+        <f t="shared" si="1"/>
         <v>240000</v>
       </c>
       <c r="J48" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="K48" s="5" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="L48" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="M48" s="5" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
     </row>
     <row r="49" spans="1:13" ht="45" x14ac:dyDescent="0.25">
@@ -3785,16 +3815,16 @@
         <v>39</v>
       </c>
       <c r="C49" s="5" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D49" s="5" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E49" s="5" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="F49" s="8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="G49" s="6">
         <v>1</v>
@@ -3803,20 +3833,20 @@
         <v>464000</v>
       </c>
       <c r="I49" s="6">
-        <f>ROUND(G49*H49,0)</f>
+        <f t="shared" si="1"/>
         <v>464000</v>
       </c>
       <c r="J49" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="K49" s="5" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="L49" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="M49" s="5" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="50" spans="1:13" ht="30" x14ac:dyDescent="0.25">
@@ -3827,16 +3857,16 @@
         <v>40</v>
       </c>
       <c r="C50" s="5" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D50" s="5" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="E50" s="5" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="F50" s="8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="G50" s="6">
         <v>1</v>
@@ -3845,20 +3875,20 @@
         <v>35990</v>
       </c>
       <c r="I50" s="6">
-        <f>ROUND(G50*H50,0)</f>
+        <f t="shared" si="1"/>
         <v>35990</v>
       </c>
       <c r="J50" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="K50" s="5" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="L50" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="M50" s="5" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
     </row>
     <row r="51" spans="1:13" ht="30" x14ac:dyDescent="0.25">
@@ -3869,16 +3899,16 @@
         <v>41</v>
       </c>
       <c r="C51" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="D51" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="D51" s="5" t="s">
+      <c r="E51" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="E51" s="5" t="s">
+      <c r="F51" s="8" t="s">
         <v>68</v>
-      </c>
-      <c r="F51" s="8" t="s">
-        <v>69</v>
       </c>
       <c r="G51" s="6">
         <v>1</v>
@@ -3887,20 +3917,20 @@
         <v>174000</v>
       </c>
       <c r="I51" s="6">
-        <f>ROUND(G51*H51,0)</f>
+        <f t="shared" si="1"/>
         <v>174000</v>
       </c>
       <c r="J51" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="K51" s="5" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="L51" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="M51" s="5" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="52" spans="1:13" ht="30" x14ac:dyDescent="0.25">
@@ -3911,38 +3941,38 @@
         <v>42</v>
       </c>
       <c r="C52" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="D52" s="5" t="s">
         <v>70</v>
       </c>
-      <c r="D52" s="5" t="s">
+      <c r="E52" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="E52" s="5" t="s">
-        <v>72</v>
-      </c>
       <c r="F52" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="G52" s="6">
-        <v>1</v>
-      </c>
-      <c r="H52" s="6">
+        <v>20</v>
+      </c>
+      <c r="G52" s="27">
+        <v>1</v>
+      </c>
+      <c r="H52" s="27">
         <v>464000</v>
       </c>
       <c r="I52" s="6">
-        <f>ROUND(G52*H52,0)</f>
+        <f t="shared" si="1"/>
         <v>464000</v>
       </c>
       <c r="J52" s="5" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="K52" s="5" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="L52" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="M52" s="5" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="53" spans="1:13" x14ac:dyDescent="0.25">
@@ -3953,16 +3983,16 @@
         <v>43</v>
       </c>
       <c r="C53" s="5" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D53" s="5" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="E53" s="5" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="F53" s="8" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G53" s="6">
         <v>2</v>
@@ -3971,20 +4001,20 @@
         <v>11600</v>
       </c>
       <c r="I53" s="6">
-        <f>ROUND(G53*H53,0)</f>
+        <f t="shared" si="1"/>
         <v>23200</v>
       </c>
       <c r="J53" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="K53" s="5" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="L53" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="M53" s="5" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="54" spans="1:13" ht="60" x14ac:dyDescent="0.25">
@@ -3995,16 +4025,16 @@
         <v>44</v>
       </c>
       <c r="C54" s="5" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D54" s="5" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="E54" s="5" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="F54" s="8" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G54" s="6">
         <v>1</v>
@@ -4013,20 +4043,20 @@
         <v>13409903</v>
       </c>
       <c r="I54" s="6">
-        <f>ROUND(G54*H54,0)</f>
+        <f t="shared" si="1"/>
         <v>13409903</v>
       </c>
       <c r="J54" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="K54" s="5" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="L54" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="M54" s="5" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="55" spans="1:13" ht="30" x14ac:dyDescent="0.25">
@@ -4037,38 +4067,38 @@
         <v>45</v>
       </c>
       <c r="C55" s="5" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D55" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="E55" s="5" t="s">
+        <v>281</v>
+      </c>
+      <c r="F55" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="G55" s="27">
+        <v>3</v>
+      </c>
+      <c r="H55" s="27">
+        <v>58000</v>
+      </c>
+      <c r="I55" s="6">
+        <f t="shared" si="1"/>
+        <v>174000</v>
+      </c>
+      <c r="J55" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="K55" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="L55" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="M55" s="5" t="s">
         <v>74</v>
-      </c>
-      <c r="E55" s="5" t="s">
-        <v>283</v>
-      </c>
-      <c r="F55" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="G55" s="6">
-        <v>3</v>
-      </c>
-      <c r="H55" s="6">
-        <v>58000</v>
-      </c>
-      <c r="I55" s="6">
-        <f>ROUND(G55*H55,0)</f>
-        <v>174000</v>
-      </c>
-      <c r="J55" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="K55" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="L55" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="M55" s="5" t="s">
-        <v>75</v>
       </c>
     </row>
     <row r="56" spans="1:13" ht="30" x14ac:dyDescent="0.25">
@@ -4079,16 +4109,16 @@
         <v>46</v>
       </c>
       <c r="C56" s="5" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D56" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="E56" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="E56" s="5" t="s">
-        <v>77</v>
-      </c>
       <c r="F56" s="8" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G56" s="6">
         <v>3</v>
@@ -4097,20 +4127,20 @@
         <v>69600</v>
       </c>
       <c r="I56" s="6">
-        <f>ROUND(G56*H56,0)</f>
+        <f t="shared" si="1"/>
         <v>208800</v>
       </c>
       <c r="J56" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="K56" s="5" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="L56" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="M56" s="5" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
     </row>
     <row r="57" spans="1:13" ht="30" x14ac:dyDescent="0.25">
@@ -4121,16 +4151,16 @@
         <v>47</v>
       </c>
       <c r="C57" s="5" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D57" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="E57" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="E57" s="5" t="s">
-        <v>79</v>
-      </c>
       <c r="F57" s="8" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G57" s="6">
         <v>3</v>
@@ -4139,20 +4169,20 @@
         <v>58000</v>
       </c>
       <c r="I57" s="6">
-        <f>ROUND(G57*H57,0)</f>
+        <f t="shared" si="1"/>
         <v>174000</v>
       </c>
       <c r="J57" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="K57" s="5" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="L57" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="M57" s="5" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="58" spans="1:13" ht="30" x14ac:dyDescent="0.25">
@@ -4163,16 +4193,16 @@
         <v>48</v>
       </c>
       <c r="C58" s="5" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D58" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="E58" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="E58" s="5" t="s">
-        <v>81</v>
-      </c>
       <c r="F58" s="8" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G58" s="6">
         <v>3</v>
@@ -4181,20 +4211,20 @@
         <v>34800</v>
       </c>
       <c r="I58" s="6">
-        <f>ROUND(G58*H58,0)</f>
+        <f t="shared" si="1"/>
         <v>104400</v>
       </c>
       <c r="J58" s="5" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="K58" s="5" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="L58" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="M58" s="5" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="59" spans="1:13" ht="30" x14ac:dyDescent="0.25">
@@ -4205,16 +4235,16 @@
         <v>49</v>
       </c>
       <c r="C59" s="5" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D59" s="5" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="E59" s="5" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="F59" s="8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="G59" s="6">
         <v>11</v>
@@ -4223,20 +4253,20 @@
         <v>2450</v>
       </c>
       <c r="I59" s="6">
-        <f>ROUND(G59*H59,0)</f>
+        <f t="shared" si="1"/>
         <v>26950</v>
       </c>
       <c r="J59" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="K59" s="5" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="L59" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="M59" s="5" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
     </row>
     <row r="60" spans="1:13" ht="30" x14ac:dyDescent="0.25">
@@ -4247,16 +4277,16 @@
         <v>50</v>
       </c>
       <c r="C60" s="5" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D60" s="5" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E60" s="5" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="F60" s="8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="G60" s="6">
         <v>1</v>
@@ -4265,20 +4295,20 @@
         <v>5990</v>
       </c>
       <c r="I60" s="6">
-        <f>ROUND(G60*H60,0)</f>
+        <f t="shared" si="1"/>
         <v>5990</v>
       </c>
       <c r="J60" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="K60" s="5" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="L60" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="M60" s="5" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
     </row>
     <row r="61" spans="1:13" ht="30" x14ac:dyDescent="0.25">
@@ -4289,16 +4319,16 @@
         <v>51</v>
       </c>
       <c r="C61" s="5" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D61" s="5" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E61" s="5" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="F61" s="8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="G61" s="6">
         <v>2</v>
@@ -4307,20 +4337,20 @@
         <v>4090</v>
       </c>
       <c r="I61" s="6">
-        <f>ROUND(G61*H61,0)</f>
+        <f t="shared" si="1"/>
         <v>8180</v>
       </c>
       <c r="J61" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="K61" s="5" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="L61" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="M61" s="5" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
     </row>
     <row r="62" spans="1:13" ht="30" x14ac:dyDescent="0.25">
@@ -4331,16 +4361,16 @@
         <v>52</v>
       </c>
       <c r="C62" s="5" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D62" s="5" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="E62" s="5" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="F62" s="8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="G62" s="6">
         <v>1</v>
@@ -4349,20 +4379,20 @@
         <v>5800</v>
       </c>
       <c r="I62" s="6">
-        <f>ROUND(G62*H62,0)</f>
+        <f t="shared" si="1"/>
         <v>5800</v>
       </c>
       <c r="J62" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="K62" s="5" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="L62" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="M62" s="5" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
     </row>
     <row r="63" spans="1:13" ht="30" x14ac:dyDescent="0.25">
@@ -4373,16 +4403,16 @@
         <v>53</v>
       </c>
       <c r="C63" s="5" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D63" s="5" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="E63" s="5" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="F63" s="8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="G63" s="6">
         <v>30</v>
@@ -4391,20 +4421,20 @@
         <v>1200</v>
       </c>
       <c r="I63" s="6">
-        <f>ROUND(G63*H63,0)</f>
+        <f t="shared" si="1"/>
         <v>36000</v>
       </c>
       <c r="J63" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="K63" s="5" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="L63" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="M63" s="5" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
     </row>
     <row r="64" spans="1:13" ht="30" x14ac:dyDescent="0.25">
@@ -4415,16 +4445,16 @@
         <v>54</v>
       </c>
       <c r="C64" s="5" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D64" s="5" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="E64" s="5" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="F64" s="8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="G64" s="6">
         <v>30</v>
@@ -4433,20 +4463,20 @@
         <v>900</v>
       </c>
       <c r="I64" s="6">
-        <f>ROUND(G64*H64,0)</f>
+        <f t="shared" si="1"/>
         <v>27000</v>
       </c>
       <c r="J64" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="K64" s="5" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="L64" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="M64" s="5" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
     </row>
     <row r="65" spans="1:13" ht="45" x14ac:dyDescent="0.25">
@@ -4457,16 +4487,16 @@
         <v>55</v>
       </c>
       <c r="C65" s="5" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D65" s="5" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E65" s="5" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="F65" s="8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="G65" s="6">
         <v>15</v>
@@ -4475,20 +4505,20 @@
         <v>1500</v>
       </c>
       <c r="I65" s="6">
-        <f>ROUND(G65*H65,0)</f>
+        <f t="shared" si="1"/>
         <v>22500</v>
       </c>
       <c r="J65" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="K65" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="K65" s="5" t="s">
-        <v>23</v>
-      </c>
       <c r="L65" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="M65" s="5" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
     </row>
     <row r="66" spans="1:13" ht="30" x14ac:dyDescent="0.25">
@@ -4499,16 +4529,16 @@
         <v>56</v>
       </c>
       <c r="C66" s="5" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D66" s="5" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="E66" s="5" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="F66" s="8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="G66" s="6">
         <v>1</v>
@@ -4517,20 +4547,20 @@
         <v>8000</v>
       </c>
       <c r="I66" s="6">
-        <f>ROUND(G66*H66,0)</f>
+        <f t="shared" si="1"/>
         <v>8000</v>
       </c>
       <c r="J66" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="K66" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="K66" s="5" t="s">
-        <v>23</v>
-      </c>
       <c r="L66" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="M66" s="5" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
     </row>
     <row r="67" spans="1:13" ht="30" x14ac:dyDescent="0.25">
@@ -4541,16 +4571,16 @@
         <v>57</v>
       </c>
       <c r="C67" s="5" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D67" s="5" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="E67" s="5" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="F67" s="8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="G67" s="6">
         <v>1</v>
@@ -4559,20 +4589,20 @@
         <v>10000</v>
       </c>
       <c r="I67" s="6">
-        <f>ROUND(G67*H67,0)</f>
+        <f t="shared" si="1"/>
         <v>10000</v>
       </c>
       <c r="J67" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="K67" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="K67" s="5" t="s">
-        <v>23</v>
-      </c>
       <c r="L67" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="M67" s="5" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
     </row>
     <row r="68" spans="1:13" ht="30" x14ac:dyDescent="0.25">
@@ -4583,16 +4613,16 @@
         <v>58</v>
       </c>
       <c r="C68" s="5" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D68" s="5" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="E68" s="5" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="F68" s="8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="G68" s="6">
         <v>1</v>
@@ -4601,20 +4631,20 @@
         <v>6000</v>
       </c>
       <c r="I68" s="6">
-        <f>ROUND(G68*H68,0)</f>
+        <f t="shared" si="1"/>
         <v>6000</v>
       </c>
       <c r="J68" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="K68" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="K68" s="5" t="s">
-        <v>23</v>
-      </c>
       <c r="L68" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="M68" s="5" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
     </row>
     <row r="69" spans="1:13" ht="30" x14ac:dyDescent="0.25">
@@ -4625,16 +4655,16 @@
         <v>59</v>
       </c>
       <c r="C69" s="5" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D69" s="5" t="s">
+        <v>91</v>
+      </c>
+      <c r="E69" s="5" t="s">
         <v>92</v>
       </c>
-      <c r="E69" s="5" t="s">
-        <v>93</v>
-      </c>
       <c r="F69" s="8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="G69" s="6">
         <v>2</v>
@@ -4643,20 +4673,20 @@
         <v>12000</v>
       </c>
       <c r="I69" s="6">
-        <f>ROUND(G69*H69,0)</f>
+        <f t="shared" si="1"/>
         <v>24000</v>
       </c>
       <c r="J69" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="K69" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="K69" s="5" t="s">
-        <v>23</v>
-      </c>
       <c r="L69" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="M69" s="5" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
     </row>
     <row r="70" spans="1:13" ht="30" x14ac:dyDescent="0.25">
@@ -4667,16 +4697,16 @@
         <v>60</v>
       </c>
       <c r="C70" s="5" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D70" s="5" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="E70" s="5" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="F70" s="8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="G70" s="6">
         <v>1</v>
@@ -4685,20 +4715,20 @@
         <v>8000</v>
       </c>
       <c r="I70" s="6">
-        <f>ROUND(G70*H70,0)</f>
+        <f t="shared" si="1"/>
         <v>8000</v>
       </c>
       <c r="J70" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="K70" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="K70" s="5" t="s">
-        <v>23</v>
-      </c>
       <c r="L70" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="M70" s="5" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
     </row>
     <row r="71" spans="1:13" ht="30" x14ac:dyDescent="0.25">
@@ -4709,16 +4739,16 @@
         <v>61</v>
       </c>
       <c r="C71" s="5" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D71" s="5" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="E71" s="5" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="F71" s="8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="G71" s="6">
         <v>3</v>
@@ -4727,20 +4757,20 @@
         <v>116000</v>
       </c>
       <c r="I71" s="6">
-        <f>ROUND(G71*H71,0)</f>
+        <f t="shared" si="1"/>
         <v>348000</v>
       </c>
       <c r="J71" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="K71" s="5" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="L71" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="M71" s="5" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="72" spans="1:13" ht="45" x14ac:dyDescent="0.25">
@@ -4751,16 +4781,16 @@
         <v>62</v>
       </c>
       <c r="C72" s="5" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D72" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E72" s="5" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="F72" s="8" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G72" s="6">
         <v>42</v>
@@ -4769,20 +4799,20 @@
         <v>8120</v>
       </c>
       <c r="I72" s="6">
-        <f>ROUND(G72*H72,0)</f>
+        <f t="shared" si="1"/>
         <v>341040</v>
       </c>
       <c r="J72" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="K72" s="5" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="L72" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="M72" s="5" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
     </row>
     <row r="73" spans="1:13" ht="30" x14ac:dyDescent="0.25">
@@ -4793,16 +4823,16 @@
         <v>63</v>
       </c>
       <c r="C73" s="5" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D73" s="5" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E73" s="5" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="F73" s="8" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G73" s="6">
         <v>9</v>
@@ -4811,20 +4841,20 @@
         <v>8700</v>
       </c>
       <c r="I73" s="6">
-        <f>ROUND(G73*H73,0)</f>
+        <f t="shared" si="1"/>
         <v>78300</v>
       </c>
       <c r="J73" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="K73" s="5" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="L73" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="M73" s="5" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
     </row>
     <row r="74" spans="1:13" ht="30" x14ac:dyDescent="0.25">
@@ -4835,16 +4865,16 @@
         <v>64</v>
       </c>
       <c r="C74" s="5" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D74" s="5" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="E74" s="5" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="F74" s="8" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G74" s="6">
         <v>6</v>
@@ -4853,20 +4883,20 @@
         <v>34800</v>
       </c>
       <c r="I74" s="6">
-        <f>ROUND(G74*H74,0)</f>
+        <f t="shared" si="1"/>
         <v>208800</v>
       </c>
       <c r="J74" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="K74" s="5" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="L74" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="M74" s="5" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
     </row>
     <row r="75" spans="1:13" ht="30" x14ac:dyDescent="0.25">
@@ -4877,16 +4907,16 @@
         <v>65</v>
       </c>
       <c r="C75" s="5" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D75" s="5" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="E75" s="5" t="s">
-        <v>290</v>
+        <v>299</v>
       </c>
       <c r="F75" s="8" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G75" s="6">
         <v>6</v>
@@ -4895,23 +4925,23 @@
         <v>9280</v>
       </c>
       <c r="I75" s="6">
-        <f>ROUND(G75*H75,0)</f>
+        <f t="shared" ref="I75:I106" si="2">ROUND(G75*H75,0)</f>
         <v>55680</v>
       </c>
       <c r="J75" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="K75" s="5" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="L75" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="M75" s="5" t="s">
-        <v>185</v>
-      </c>
-    </row>
-    <row r="76" spans="1:13" ht="45" x14ac:dyDescent="0.25">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="76" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A76" s="8">
         <v>1</v>
       </c>
@@ -4919,16 +4949,16 @@
         <v>66</v>
       </c>
       <c r="C76" s="5" t="s">
-        <v>66</v>
-      </c>
-      <c r="D76" s="5" t="s">
-        <v>186</v>
-      </c>
-      <c r="E76" s="5" t="s">
-        <v>291</v>
+        <v>65</v>
+      </c>
+      <c r="D76" s="25" t="s">
+        <v>185</v>
+      </c>
+      <c r="E76" s="25" t="s">
+        <v>300</v>
       </c>
       <c r="F76" s="8" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G76" s="6">
         <v>1</v>
@@ -4937,20 +4967,20 @@
         <v>2731613</v>
       </c>
       <c r="I76" s="6">
-        <f>ROUND(G76*H76,0)</f>
+        <f t="shared" si="2"/>
         <v>2731613</v>
       </c>
       <c r="J76" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="K76" s="5" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="L76" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="M76" s="5" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
     </row>
     <row r="77" spans="1:13" ht="45" x14ac:dyDescent="0.25">
@@ -4961,16 +4991,16 @@
         <v>67</v>
       </c>
       <c r="C77" s="5" t="s">
-        <v>66</v>
-      </c>
-      <c r="D77" s="5" t="s">
-        <v>188</v>
-      </c>
-      <c r="E77" s="5" t="s">
-        <v>292</v>
+        <v>65</v>
+      </c>
+      <c r="D77" s="25" t="s">
+        <v>301</v>
+      </c>
+      <c r="E77" s="25" t="s">
+        <v>288</v>
       </c>
       <c r="F77" s="8" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G77" s="6">
         <v>1</v>
@@ -4979,20 +5009,20 @@
         <v>1912129</v>
       </c>
       <c r="I77" s="6">
-        <f>ROUND(G77*H77,0)</f>
+        <f t="shared" si="2"/>
         <v>1912129</v>
       </c>
       <c r="J77" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="K77" s="5" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="L77" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="M77" s="5" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
     </row>
     <row r="78" spans="1:13" ht="45" x14ac:dyDescent="0.25">
@@ -5003,16 +5033,16 @@
         <v>68</v>
       </c>
       <c r="C78" s="5" t="s">
-        <v>66</v>
-      </c>
-      <c r="D78" s="5" t="s">
-        <v>189</v>
+        <v>65</v>
+      </c>
+      <c r="D78" s="24" t="s">
+        <v>187</v>
       </c>
       <c r="E78" s="5" t="s">
-        <v>293</v>
+        <v>289</v>
       </c>
       <c r="F78" s="8" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G78" s="6">
         <v>1</v>
@@ -5021,20 +5051,20 @@
         <v>2731613</v>
       </c>
       <c r="I78" s="6">
-        <f>ROUND(G78*H78,0)</f>
+        <f t="shared" si="2"/>
         <v>2731613</v>
       </c>
       <c r="J78" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="K78" s="5" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="L78" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="M78" s="5" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
     </row>
     <row r="79" spans="1:13" ht="30" x14ac:dyDescent="0.25">
@@ -5045,16 +5075,16 @@
         <v>69</v>
       </c>
       <c r="C79" s="5" t="s">
-        <v>66</v>
-      </c>
-      <c r="D79" s="5" t="s">
-        <v>190</v>
+        <v>65</v>
+      </c>
+      <c r="D79" s="24" t="s">
+        <v>188</v>
       </c>
       <c r="E79" s="5" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="F79" s="8" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G79" s="6">
         <v>1</v>
@@ -5063,20 +5093,20 @@
         <v>2320000</v>
       </c>
       <c r="I79" s="6">
-        <f>ROUND(G79*H79,0)</f>
+        <f t="shared" si="2"/>
         <v>2320000</v>
       </c>
       <c r="J79" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="K79" s="5" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="L79" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="M79" s="5" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
     </row>
     <row r="80" spans="1:13" ht="30" x14ac:dyDescent="0.25">
@@ -5087,16 +5117,16 @@
         <v>70</v>
       </c>
       <c r="C80" s="5" t="s">
-        <v>66</v>
-      </c>
-      <c r="D80" s="5" t="s">
-        <v>191</v>
+        <v>65</v>
+      </c>
+      <c r="D80" s="24" t="s">
+        <v>189</v>
       </c>
       <c r="E80" s="5" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="F80" s="8" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G80" s="6">
         <v>1</v>
@@ -5105,20 +5135,20 @@
         <v>1624000</v>
       </c>
       <c r="I80" s="6">
-        <f>ROUND(G80*H80,0)</f>
+        <f t="shared" si="2"/>
         <v>1624000</v>
       </c>
       <c r="J80" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="K80" s="5" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="L80" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="M80" s="5" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
     </row>
     <row r="81" spans="1:13" ht="30" x14ac:dyDescent="0.25">
@@ -5129,16 +5159,16 @@
         <v>71</v>
       </c>
       <c r="C81" s="5" t="s">
-        <v>66</v>
-      </c>
-      <c r="D81" s="5" t="s">
-        <v>192</v>
+        <v>65</v>
+      </c>
+      <c r="D81" s="24" t="s">
+        <v>190</v>
       </c>
       <c r="E81" s="5" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="F81" s="8" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G81" s="6">
         <v>1</v>
@@ -5147,20 +5177,20 @@
         <v>1624000</v>
       </c>
       <c r="I81" s="6">
-        <f>ROUND(G81*H81,0)</f>
+        <f t="shared" si="2"/>
         <v>1624000</v>
       </c>
       <c r="J81" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="K81" s="5" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="L81" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="M81" s="5" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
     </row>
     <row r="82" spans="1:13" ht="30" x14ac:dyDescent="0.25">
@@ -5171,16 +5201,16 @@
         <v>72</v>
       </c>
       <c r="C82" s="5" t="s">
-        <v>66</v>
-      </c>
-      <c r="D82" s="5" t="s">
-        <v>193</v>
+        <v>65</v>
+      </c>
+      <c r="D82" s="24" t="s">
+        <v>191</v>
       </c>
       <c r="E82" s="5" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="F82" s="8" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G82" s="6">
         <v>1</v>
@@ -5189,20 +5219,20 @@
         <v>1624000</v>
       </c>
       <c r="I82" s="6">
-        <f>ROUND(G82*H82,0)</f>
+        <f t="shared" si="2"/>
         <v>1624000</v>
       </c>
       <c r="J82" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="K82" s="5" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="L82" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="M82" s="5" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
     </row>
     <row r="83" spans="1:13" ht="30" x14ac:dyDescent="0.25">
@@ -5213,16 +5243,16 @@
         <v>73</v>
       </c>
       <c r="C83" s="5" t="s">
-        <v>66</v>
-      </c>
-      <c r="D83" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="D83" s="26" t="s">
+        <v>99</v>
+      </c>
+      <c r="E83" s="5" t="s">
         <v>100</v>
       </c>
-      <c r="E83" s="5" t="s">
-        <v>101</v>
-      </c>
       <c r="F83" s="8" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G83" s="6">
         <v>1</v>
@@ -5231,20 +5261,20 @@
         <v>2320000</v>
       </c>
       <c r="I83" s="6">
-        <f>ROUND(G83*H83,0)</f>
+        <f t="shared" si="2"/>
         <v>2320000</v>
       </c>
       <c r="J83" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="K83" s="5" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="L83" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="M83" s="5" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="84" spans="1:13" ht="30" x14ac:dyDescent="0.25">
@@ -5255,16 +5285,16 @@
         <v>74</v>
       </c>
       <c r="C84" s="5" t="s">
-        <v>66</v>
-      </c>
-      <c r="D84" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="D84" s="26" t="s">
+        <v>101</v>
+      </c>
+      <c r="E84" s="5" t="s">
         <v>102</v>
       </c>
-      <c r="E84" s="5" t="s">
-        <v>103</v>
-      </c>
       <c r="F84" s="8" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G84" s="6">
         <v>1</v>
@@ -5273,20 +5303,20 @@
         <v>522000</v>
       </c>
       <c r="I84" s="6">
-        <f>ROUND(G84*H84,0)</f>
+        <f t="shared" si="2"/>
         <v>522000</v>
       </c>
       <c r="J84" s="5" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="K84" s="5" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="L84" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="M84" s="5" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
     </row>
     <row r="85" spans="1:13" ht="30" x14ac:dyDescent="0.25">
@@ -5297,16 +5327,16 @@
         <v>75</v>
       </c>
       <c r="C85" s="5" t="s">
-        <v>66</v>
-      </c>
-      <c r="D85" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="D85" s="26" t="s">
+        <v>103</v>
+      </c>
+      <c r="E85" s="5" t="s">
         <v>104</v>
       </c>
-      <c r="E85" s="5" t="s">
-        <v>105</v>
-      </c>
       <c r="F85" s="8" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G85" s="6">
         <v>3</v>
@@ -5315,20 +5345,20 @@
         <v>29000</v>
       </c>
       <c r="I85" s="6">
-        <f>ROUND(G85*H85,0)</f>
+        <f t="shared" si="2"/>
         <v>87000</v>
       </c>
       <c r="J85" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="K85" s="5" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="L85" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="M85" s="5" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="86" spans="1:13" ht="30" x14ac:dyDescent="0.25">
@@ -5339,16 +5369,16 @@
         <v>76</v>
       </c>
       <c r="C86" s="5" t="s">
-        <v>66</v>
-      </c>
-      <c r="D86" s="5" t="s">
-        <v>252</v>
+        <v>65</v>
+      </c>
+      <c r="D86" s="26" t="s">
+        <v>250</v>
       </c>
       <c r="E86" s="5" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="F86" s="8" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G86" s="6">
         <v>1</v>
@@ -5357,20 +5387,20 @@
         <v>58000</v>
       </c>
       <c r="I86" s="6">
-        <f>ROUND(G86*H86,0)</f>
+        <f t="shared" si="2"/>
         <v>58000</v>
       </c>
       <c r="J86" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="K86" s="5" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="L86" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="M86" s="5" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="87" spans="1:13" ht="30" x14ac:dyDescent="0.25">
@@ -5381,16 +5411,16 @@
         <v>77</v>
       </c>
       <c r="C87" s="5" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D87" s="5" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="E87" s="5" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="F87" s="8" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G87" s="6">
         <v>1</v>
@@ -5399,20 +5429,20 @@
         <v>25000</v>
       </c>
       <c r="I87" s="6">
-        <f>ROUND(G87*H87,0)</f>
+        <f t="shared" si="2"/>
         <v>25000</v>
       </c>
       <c r="J87" s="5" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="K87" s="5" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="L87" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="M87" s="5" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
     </row>
     <row r="88" spans="1:13" ht="45" x14ac:dyDescent="0.25">
@@ -5423,16 +5453,16 @@
         <v>78</v>
       </c>
       <c r="C88" s="5" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D88" s="5" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="E88" s="5" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="F88" s="8" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G88" s="6">
         <v>1</v>
@@ -5441,20 +5471,20 @@
         <v>500000</v>
       </c>
       <c r="I88" s="6">
-        <f>ROUND(G88*H88,0)</f>
+        <f t="shared" si="2"/>
         <v>500000</v>
       </c>
       <c r="J88" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="K88" s="5" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="L88" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="M88" s="5" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
     </row>
     <row r="89" spans="1:13" ht="45" x14ac:dyDescent="0.25">
@@ -5465,16 +5495,16 @@
         <v>79</v>
       </c>
       <c r="C89" s="5" t="s">
+        <v>255</v>
+      </c>
+      <c r="D89" s="26" t="s">
+        <v>256</v>
+      </c>
+      <c r="E89" s="5" t="s">
         <v>257</v>
       </c>
-      <c r="D89" s="5" t="s">
+      <c r="F89" s="8" t="s">
         <v>258</v>
-      </c>
-      <c r="E89" s="5" t="s">
-        <v>259</v>
-      </c>
-      <c r="F89" s="8" t="s">
-        <v>260</v>
       </c>
       <c r="G89" s="6">
         <v>1</v>
@@ -5483,20 +5513,20 @@
         <v>87404855</v>
       </c>
       <c r="I89" s="6">
-        <f>ROUND(G89*H89,0)</f>
+        <f t="shared" si="2"/>
         <v>87404855</v>
       </c>
       <c r="J89" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="K89" s="5" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="L89" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="M89" s="5" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
     </row>
     <row r="90" spans="1:13" ht="45" x14ac:dyDescent="0.25">
@@ -5507,16 +5537,16 @@
         <v>80</v>
       </c>
       <c r="C90" s="5" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D90" s="5" t="s">
+        <v>109</v>
+      </c>
+      <c r="E90" s="5" t="s">
+        <v>260</v>
+      </c>
+      <c r="F90" s="8" t="s">
         <v>110</v>
-      </c>
-      <c r="E90" s="5" t="s">
-        <v>262</v>
-      </c>
-      <c r="F90" s="8" t="s">
-        <v>111</v>
       </c>
       <c r="G90" s="6">
         <v>1</v>
@@ -5525,20 +5555,20 @@
         <v>2141129</v>
       </c>
       <c r="I90" s="6">
-        <f>ROUND(G90*H90,0)</f>
+        <f t="shared" si="2"/>
         <v>2141129</v>
       </c>
       <c r="J90" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="K90" s="5" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="L90" s="5" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="M90" s="5" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
     </row>
     <row r="91" spans="1:13" x14ac:dyDescent="0.25">
@@ -5546,7 +5576,7 @@
       <c r="B91" s="9"/>
       <c r="C91" s="4"/>
       <c r="D91" s="4" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="E91" s="4"/>
       <c r="F91" s="9"/>
@@ -5586,267 +5616,267 @@
   <sheetData>
     <row r="1" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>294</v>
+        <v>290</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>295</v>
+        <v>291</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="10" t="s">
+        <v>117</v>
+      </c>
+      <c r="B4" s="10" t="s">
         <v>118</v>
       </c>
-      <c r="B4" s="10" t="s">
+      <c r="C4" s="10" t="s">
         <v>119</v>
       </c>
-      <c r="C4" s="10" t="s">
+      <c r="D4" s="10" t="s">
         <v>120</v>
       </c>
-      <c r="D4" s="10" t="s">
+      <c r="E4" s="10" t="s">
         <v>121</v>
-      </c>
-      <c r="E4" s="10" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A5" s="11" t="s">
+        <v>122</v>
+      </c>
+      <c r="B5" s="11" t="s">
         <v>123</v>
-      </c>
-      <c r="B5" s="11" t="s">
-        <v>124</v>
       </c>
       <c r="C5" s="12">
         <v>2450</v>
       </c>
       <c r="D5" s="11" t="s">
+        <v>124</v>
+      </c>
+      <c r="E5" s="11" t="s">
         <v>125</v>
-      </c>
-      <c r="E5" s="11" t="s">
-        <v>126</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A6" s="11" t="s">
+        <v>126</v>
+      </c>
+      <c r="B6" s="11" t="s">
         <v>127</v>
-      </c>
-      <c r="B6" s="11" t="s">
-        <v>128</v>
       </c>
       <c r="C6" s="12">
         <v>2150</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E6" s="11" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A7" s="11" t="s">
+        <v>129</v>
+      </c>
+      <c r="B7" s="11" t="s">
         <v>130</v>
-      </c>
-      <c r="B7" s="11" t="s">
-        <v>131</v>
       </c>
       <c r="C7" s="12">
         <v>5990</v>
       </c>
       <c r="D7" s="11" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E7" s="11" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A8" s="11" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>296</v>
+        <v>292</v>
       </c>
       <c r="C8" s="12">
         <v>2155</v>
       </c>
       <c r="D8" s="11" t="s">
+        <v>133</v>
+      </c>
+      <c r="E8" s="11" t="s">
         <v>134</v>
-      </c>
-      <c r="E8" s="11" t="s">
-        <v>135</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" s="11" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>297</v>
+        <v>293</v>
       </c>
       <c r="C9" s="12">
         <v>35</v>
       </c>
       <c r="D9" s="11" t="s">
+        <v>136</v>
+      </c>
+      <c r="E9" s="11" t="s">
         <v>137</v>
-      </c>
-      <c r="E9" s="11" t="s">
-        <v>138</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A10" s="11" t="s">
+        <v>138</v>
+      </c>
+      <c r="B10" s="11" t="s">
         <v>139</v>
-      </c>
-      <c r="B10" s="11" t="s">
-        <v>140</v>
       </c>
       <c r="C10" s="12">
         <v>190</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="E10" s="11" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="11" t="s">
+        <v>141</v>
+      </c>
+      <c r="B11" s="11" t="s">
         <v>142</v>
-      </c>
-      <c r="B11" s="11" t="s">
-        <v>143</v>
       </c>
       <c r="C11" s="12">
         <v>1019</v>
       </c>
       <c r="D11" s="11" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="E11" s="11" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="11" t="s">
+        <v>144</v>
+      </c>
+      <c r="B12" s="11" t="s">
         <v>145</v>
-      </c>
-      <c r="B12" s="11" t="s">
-        <v>146</v>
       </c>
       <c r="C12" s="12">
         <v>14</v>
       </c>
       <c r="D12" s="11" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="E12" s="11" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A13" s="11" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B13" s="11" t="s">
-        <v>298</v>
+        <v>294</v>
       </c>
       <c r="C13" s="12">
         <v>680</v>
       </c>
       <c r="D13" s="11" t="s">
+        <v>148</v>
+      </c>
+      <c r="E13" s="11" t="s">
         <v>149</v>
-      </c>
-      <c r="E13" s="11" t="s">
-        <v>150</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A14" s="11" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B14" s="11" t="s">
-        <v>299</v>
+        <v>295</v>
       </c>
       <c r="C14" s="12">
         <v>165</v>
       </c>
       <c r="D14" s="11" t="s">
+        <v>151</v>
+      </c>
+      <c r="E14" s="11" t="s">
         <v>152</v>
-      </c>
-      <c r="E14" s="11" t="s">
-        <v>153</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A15" s="11" t="s">
+        <v>153</v>
+      </c>
+      <c r="B15" s="11" t="s">
         <v>154</v>
-      </c>
-      <c r="B15" s="11" t="s">
-        <v>155</v>
       </c>
       <c r="C15" s="12">
         <v>560</v>
       </c>
       <c r="D15" s="11" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="E15" s="11" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="11" t="s">
+        <v>156</v>
+      </c>
+      <c r="B16" s="11" t="s">
         <v>157</v>
-      </c>
-      <c r="B16" s="11" t="s">
-        <v>158</v>
       </c>
       <c r="C16" s="12">
         <v>661</v>
       </c>
       <c r="D16" s="11" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="E16" s="11" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A17" s="11" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B17" s="11" t="s">
-        <v>300</v>
+        <v>296</v>
       </c>
       <c r="C17" s="12">
         <v>285</v>
       </c>
       <c r="D17" s="11" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="E17" s="11" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A18" s="11" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B18" s="11" t="s">
-        <v>301</v>
+        <v>297</v>
       </c>
       <c r="C18" s="12">
         <v>3395</v>
       </c>
       <c r="D18" s="11" t="s">
+        <v>162</v>
+      </c>
+      <c r="E18" s="11" t="s">
         <v>163</v>
-      </c>
-      <c r="E18" s="11" t="s">
-        <v>164</v>
       </c>
     </row>
   </sheetData>

</xml_diff>